<commit_message>
data(gbp): daily refresh 2026-09-17T15:11Z
</commit_message>
<xml_diff>
--- a/logs/gbp/raw/boe_str.xlsx
+++ b/logs/gbp/raw/boe_str.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bankofenglandcouk.sharepoint.com/sites/SMD-Ops/Shared Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="106" documentId="11_5C6355D4097423DEAD7C7E3551DBF34CECDC700E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9A40A9E-8D8B-4D81-9A67-C376DA55F733}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{527CADD2-1457-4860-B3BA-B939FAC6090C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-16200" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" ST OMO Summary" sheetId="1" r:id="rId1"/>
@@ -277,10 +277,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -571,7 +567,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:H204"/>
+  <dimension ref="A1:H205"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" style="1" customWidth="1"/>
@@ -4085,6 +4081,23 @@
         <v>0</v>
       </c>
     </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A205" s="2">
+        <v>46282</v>
+      </c>
+      <c r="B205" s="3">
+        <v>7</v>
+      </c>
+      <c r="C205" s="2">
+        <v>46289</v>
+      </c>
+      <c r="D205" s="23">
+        <v>125390</v>
+      </c>
+      <c r="E205" s="24">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.98425196850393704" right="0.98425196850393704" top="0.98425196850393704" bottom="1.9842519685039399" header="0.98425196850393704" footer="0.98425196850393704"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
data(gbp): daily refresh 2026-09-24T15:23Z
</commit_message>
<xml_diff>
--- a/logs/gbp/raw/boe_str.xlsx
+++ b/logs/gbp/raw/boe_str.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bankofenglandcouk.sharepoint.com/sites/SMD-Ops/Shared Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{527CADD2-1457-4860-B3BA-B939FAC6090C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="6_{6357EF7E-F4D8-4EEB-8998-019A4B55854A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAD262A6-6FB8-4B53-9F6F-A2BFB8699E38}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-16200" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" ST OMO Summary" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
     <numFmt numFmtId="165" formatCode="[$-10409]0.0"/>
     <numFmt numFmtId="166" formatCode="[$-10409]0.00"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -160,6 +160,11 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -181,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -260,6 +265,18 @@
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -567,7 +584,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:H205"/>
+  <dimension ref="A1:H206"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" style="1" customWidth="1"/>
@@ -4098,6 +4115,23 @@
         <v>0</v>
       </c>
     </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A206" s="26">
+        <v>46289</v>
+      </c>
+      <c r="B206" s="27">
+        <v>7</v>
+      </c>
+      <c r="C206" s="26">
+        <v>46296</v>
+      </c>
+      <c r="D206" s="28">
+        <v>128918</v>
+      </c>
+      <c r="E206" s="29">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.98425196850393704" right="0.98425196850393704" top="0.98425196850393704" bottom="1.9842519685039399" header="0.98425196850393704" footer="0.98425196850393704"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
data(gbp): daily refresh 2026-10-02T16:20Z
</commit_message>
<xml_diff>
--- a/logs/gbp/raw/boe_str.xlsx
+++ b/logs/gbp/raw/boe_str.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bankofenglandcouk.sharepoint.com/sites/SMD-Ops/Shared Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="6_{6357EF7E-F4D8-4EEB-8998-019A4B55854A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAD262A6-6FB8-4B53-9F6F-A2BFB8699E38}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3CD4B90-E5C6-40FE-98A0-07A0D2812822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30" yWindow="-16200" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" ST OMO Summary" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
     <numFmt numFmtId="165" formatCode="[$-10409]0.0"/>
     <numFmt numFmtId="166" formatCode="[$-10409]0.00"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -164,6 +164,13 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -186,7 +193,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -279,6 +286,7 @@
     <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -584,7 +592,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:H206"/>
+  <dimension ref="A1:H207"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" style="1" customWidth="1"/>
@@ -3894,7 +3902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A193" s="21">
         <v>46198</v>
       </c>
@@ -3911,7 +3919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A194" s="21">
         <v>46205</v>
       </c>
@@ -3928,7 +3936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A195" s="21">
         <v>46212</v>
       </c>
@@ -3945,7 +3953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A196" s="21">
         <v>46219</v>
       </c>
@@ -3962,7 +3970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A197" s="21">
         <v>46226</v>
       </c>
@@ -3979,7 +3987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A198" s="21">
         <v>46233</v>
       </c>
@@ -3996,7 +4004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A199" s="21">
         <v>46240</v>
       </c>
@@ -4013,7 +4021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A200" s="21">
         <v>46247</v>
       </c>
@@ -4030,7 +4038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A201" s="21">
         <v>46254</v>
       </c>
@@ -4047,7 +4055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A202" s="21">
         <v>46261</v>
       </c>
@@ -4064,7 +4072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A203" s="2">
         <v>46268</v>
       </c>
@@ -4081,7 +4089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A204" s="21">
         <v>46275</v>
       </c>
@@ -4098,7 +4106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A205" s="2">
         <v>46282</v>
       </c>
@@ -4115,7 +4123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A206" s="26">
         <v>46289</v>
       </c>
@@ -4131,6 +4139,26 @@
       <c r="E206" s="29">
         <v>0</v>
       </c>
+    </row>
+    <row r="207" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A207" s="26">
+        <v>46296</v>
+      </c>
+      <c r="B207" s="27">
+        <v>7</v>
+      </c>
+      <c r="C207" s="26">
+        <v>46303</v>
+      </c>
+      <c r="D207" s="28">
+        <v>133441</v>
+      </c>
+      <c r="E207" s="29">
+        <v>0</v>
+      </c>
+      <c r="F207" s="30"/>
+      <c r="G207" s="30"/>
+      <c r="H207" s="30"/>
     </row>
   </sheetData>
   <pageMargins left="0.98425196850393704" right="0.98425196850393704" top="0.98425196850393704" bottom="1.9842519685039399" header="0.98425196850393704" footer="0.98425196850393704"/>

</xml_diff>

<commit_message>
data(gbp): daily refresh 2026-10-08T17:30Z
</commit_message>
<xml_diff>
--- a/logs/gbp/raw/boe_str.xlsx
+++ b/logs/gbp/raw/boe_str.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bankofenglandcouk.sharepoint.com/sites/SMD-Ops/Shared Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3CD4B90-E5C6-40FE-98A0-07A0D2812822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B9531BF-D910-4BB3-9CE9-343879D47386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30" yWindow="-16200" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-16200" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" ST OMO Summary" sheetId="1" r:id="rId1"/>
@@ -592,7 +592,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:H207"/>
+  <dimension ref="A1:H208"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" style="1" customWidth="1"/>
@@ -4160,6 +4160,23 @@
       <c r="G207" s="30"/>
       <c r="H207" s="30"/>
     </row>
+    <row r="208" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A208" s="2">
+        <v>46303</v>
+      </c>
+      <c r="B208" s="27">
+        <v>7</v>
+      </c>
+      <c r="C208" s="2">
+        <v>46310</v>
+      </c>
+      <c r="D208" s="28">
+        <v>132102</v>
+      </c>
+      <c r="E208" s="29">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.98425196850393704" right="0.98425196850393704" top="0.98425196850393704" bottom="1.9842519685039399" header="0.98425196850393704" footer="0.98425196850393704"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
data(gbp): daily refresh 2026-10-15T15:13Z
</commit_message>
<xml_diff>
--- a/logs/gbp/raw/boe_str.xlsx
+++ b/logs/gbp/raw/boe_str.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30610"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bankofenglandcouk.sharepoint.com/sites/SMD-Ops/Shared Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B9531BF-D910-4BB3-9CE9-343879D47386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="6_{6357EF7E-F4D8-4EEB-8998-019A4B55854A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4039A544-9F63-40C1-8E4D-C2F4F752A111}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-16200" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" ST OMO Summary" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
     <numFmt numFmtId="165" formatCode="[$-10409]0.0"/>
     <numFmt numFmtId="166" formatCode="[$-10409]0.00"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -162,12 +162,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -193,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -274,19 +268,7 @@
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -592,26 +574,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:H208"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:H209"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="17.54296875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.453125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.54296875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="24.1796875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="35.453125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="9.1796875" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.81640625" style="1"/>
+    <col min="1" max="1" width="17.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="24.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="35.42578125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="13.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="13.7" customHeight="1">
       <c r="A1"/>
       <c r="B1"/>
       <c r="C1"/>
       <c r="D1"/>
       <c r="E1"/>
     </row>
-    <row r="2" spans="1:5" ht="42" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="42">
       <c r="A2" s="20" t="s">
         <v>0</v>
       </c>
@@ -628,7 +610,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5">
       <c r="A3" s="21">
         <v>44840</v>
       </c>
@@ -645,7 +627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5">
       <c r="A4" s="21">
         <v>44847</v>
       </c>
@@ -662,7 +644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5">
       <c r="A5" s="21">
         <v>44854</v>
       </c>
@@ -679,7 +661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5">
       <c r="A6" s="21">
         <v>44861</v>
       </c>
@@ -696,7 +678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5">
       <c r="A7" s="21">
         <v>44868</v>
       </c>
@@ -713,7 +695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5">
       <c r="A8" s="21">
         <v>44875</v>
       </c>
@@ -730,7 +712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5">
       <c r="A9" s="21">
         <v>44882</v>
       </c>
@@ -747,7 +729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5">
       <c r="A10" s="21">
         <v>44889</v>
       </c>
@@ -764,7 +746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5">
       <c r="A11" s="21">
         <v>44896</v>
       </c>
@@ -781,7 +763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5">
       <c r="A12" s="21">
         <v>44903</v>
       </c>
@@ -798,7 +780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5">
       <c r="A13" s="21">
         <v>44910</v>
       </c>
@@ -815,7 +797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5">
       <c r="A14" s="21">
         <v>44917</v>
       </c>
@@ -832,7 +814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5">
       <c r="A15" s="21">
         <v>44931</v>
       </c>
@@ -849,7 +831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5">
       <c r="A16" s="21">
         <v>44938</v>
       </c>
@@ -866,7 +848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5">
       <c r="A17" s="21">
         <v>44945</v>
       </c>
@@ -883,7 +865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5">
       <c r="A18" s="21">
         <v>44952</v>
       </c>
@@ -900,7 +882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5">
       <c r="A19" s="21">
         <v>44959</v>
       </c>
@@ -917,7 +899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5">
       <c r="A20" s="21">
         <v>44966</v>
       </c>
@@ -934,7 +916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5">
       <c r="A21" s="21">
         <v>44973</v>
       </c>
@@ -951,7 +933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5">
       <c r="A22" s="21">
         <v>44980</v>
       </c>
@@ -968,7 +950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5">
       <c r="A23" s="21">
         <v>44987</v>
       </c>
@@ -985,7 +967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5">
       <c r="A24" s="21">
         <v>44994</v>
       </c>
@@ -1002,7 +984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5">
       <c r="A25" s="21">
         <v>45001</v>
       </c>
@@ -1019,7 +1001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5">
       <c r="A26" s="21">
         <v>45008</v>
       </c>
@@ -1036,7 +1018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5">
       <c r="A27" s="21">
         <v>45015</v>
       </c>
@@ -1053,7 +1035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5">
       <c r="A28" s="21">
         <v>45022</v>
       </c>
@@ -1070,7 +1052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5">
       <c r="A29" s="21">
         <v>45029</v>
       </c>
@@ -1087,7 +1069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5">
       <c r="A30" s="21">
         <v>45036</v>
       </c>
@@ -1104,7 +1086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5">
       <c r="A31" s="21">
         <v>45043</v>
       </c>
@@ -1121,7 +1103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5">
       <c r="A32" s="21">
         <v>45050</v>
       </c>
@@ -1138,7 +1120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5">
       <c r="A33" s="21">
         <v>45057</v>
       </c>
@@ -1155,7 +1137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5">
       <c r="A34" s="21">
         <v>45064</v>
       </c>
@@ -1172,7 +1154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5">
       <c r="A35" s="21">
         <v>45071</v>
       </c>
@@ -1189,7 +1171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5">
       <c r="A36" s="21">
         <v>45078</v>
       </c>
@@ -1206,7 +1188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5">
       <c r="A37" s="21">
         <v>45085</v>
       </c>
@@ -1223,7 +1205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5">
       <c r="A38" s="21">
         <v>45092</v>
       </c>
@@ -1240,7 +1222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5">
       <c r="A39" s="21">
         <v>45099</v>
       </c>
@@ -1257,7 +1239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5">
       <c r="A40" s="21">
         <v>45106</v>
       </c>
@@ -1274,7 +1256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5">
       <c r="A41" s="21">
         <v>45113</v>
       </c>
@@ -1291,7 +1273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5">
       <c r="A42" s="21">
         <v>45120</v>
       </c>
@@ -1308,7 +1290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5">
       <c r="A43" s="21">
         <v>45127</v>
       </c>
@@ -1325,7 +1307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5">
       <c r="A44" s="21">
         <v>45134</v>
       </c>
@@ -1342,7 +1324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5">
       <c r="A45" s="21">
         <v>45141</v>
       </c>
@@ -1359,7 +1341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5">
       <c r="A46" s="21">
         <v>45148</v>
       </c>
@@ -1376,7 +1358,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5">
       <c r="A47" s="21">
         <v>45155</v>
       </c>
@@ -1393,7 +1375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5">
       <c r="A48" s="21">
         <v>45162</v>
       </c>
@@ -1410,7 +1392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5">
       <c r="A49" s="21">
         <v>45169</v>
       </c>
@@ -1427,7 +1409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5">
       <c r="A50" s="21">
         <v>45176</v>
       </c>
@@ -1444,7 +1426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5">
       <c r="A51" s="21">
         <v>45183</v>
       </c>
@@ -1461,7 +1443,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5">
       <c r="A52" s="21">
         <v>45190</v>
       </c>
@@ -1478,7 +1460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5">
       <c r="A53" s="21">
         <v>45197</v>
       </c>
@@ -1495,7 +1477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5">
       <c r="A54" s="21">
         <v>45204</v>
       </c>
@@ -1512,7 +1494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5">
       <c r="A55" s="21">
         <v>45211</v>
       </c>
@@ -1529,7 +1511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5">
       <c r="A56" s="21">
         <v>45218</v>
       </c>
@@ -1546,7 +1528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5">
       <c r="A57" s="21">
         <v>45225</v>
       </c>
@@ -1563,7 +1545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5">
       <c r="A58" s="21">
         <v>45232</v>
       </c>
@@ -1580,7 +1562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5">
       <c r="A59" s="21">
         <v>45239</v>
       </c>
@@ -1597,7 +1579,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" s="6" customFormat="1">
       <c r="A60" s="21">
         <v>45246</v>
       </c>
@@ -1614,7 +1596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5">
       <c r="A61" s="21">
         <v>45253</v>
       </c>
@@ -1631,7 +1613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5">
       <c r="A62" s="21">
         <v>45260</v>
       </c>
@@ -1648,7 +1630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5">
       <c r="A63" s="21">
         <v>45267</v>
       </c>
@@ -1665,7 +1647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" s="6" customFormat="1">
       <c r="A64" s="21">
         <v>45274</v>
       </c>
@@ -1682,7 +1664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5">
       <c r="A65" s="21">
         <v>45281</v>
       </c>
@@ -1699,7 +1681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" s="6" customFormat="1">
       <c r="A66" s="21">
         <v>45295</v>
       </c>
@@ -1716,7 +1698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5">
       <c r="A67" s="21">
         <v>45302</v>
       </c>
@@ -1733,7 +1715,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5">
       <c r="A68" s="21">
         <v>45309</v>
       </c>
@@ -1750,7 +1732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5">
       <c r="A69" s="21">
         <v>45316</v>
       </c>
@@ -1767,7 +1749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" s="7" customFormat="1">
       <c r="A70" s="21">
         <v>45323</v>
       </c>
@@ -1784,7 +1766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" s="7" customFormat="1">
       <c r="A71" s="21">
         <v>45330</v>
       </c>
@@ -1801,7 +1783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" s="7" customFormat="1">
       <c r="A72" s="21">
         <v>45337</v>
       </c>
@@ -1818,7 +1800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5">
       <c r="A73" s="21">
         <v>45344</v>
       </c>
@@ -1835,7 +1817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" s="7" customFormat="1">
       <c r="A74" s="21">
         <v>45351</v>
       </c>
@@ -1852,7 +1834,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5">
       <c r="A75" s="21">
         <v>45358</v>
       </c>
@@ -1869,7 +1851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5">
       <c r="A76" s="21">
         <v>45365</v>
       </c>
@@ -1886,7 +1868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5">
       <c r="A77" s="21">
         <v>45372</v>
       </c>
@@ -1903,7 +1885,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5">
       <c r="A78" s="21">
         <v>45379</v>
       </c>
@@ -1920,7 +1902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5">
       <c r="A79" s="21">
         <v>45386</v>
       </c>
@@ -1937,7 +1919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5">
       <c r="A80" s="21">
         <v>45393</v>
       </c>
@@ -1954,7 +1936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5">
       <c r="A81" s="21">
         <v>45400</v>
       </c>
@@ -1971,7 +1953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5">
       <c r="A82" s="21">
         <v>45407</v>
       </c>
@@ -1988,7 +1970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5">
       <c r="A83" s="21">
         <v>45414</v>
       </c>
@@ -2005,7 +1987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" s="8" customFormat="1">
       <c r="A84" s="21">
         <v>45421</v>
       </c>
@@ -2022,7 +2004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5">
       <c r="A85" s="21">
         <v>45428</v>
       </c>
@@ -2039,7 +2021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" s="8" customFormat="1">
       <c r="A86" s="21">
         <v>45435</v>
       </c>
@@ -2056,7 +2038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5">
       <c r="A87" s="21">
         <v>45442</v>
       </c>
@@ -2073,7 +2055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5">
       <c r="A88" s="21">
         <v>45449</v>
       </c>
@@ -2090,7 +2072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5">
       <c r="A89" s="21">
         <v>45456</v>
       </c>
@@ -2107,7 +2089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5">
       <c r="A90" s="21">
         <v>45463</v>
       </c>
@@ -2124,7 +2106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5">
       <c r="A91" s="21">
         <v>45470</v>
       </c>
@@ -2141,7 +2123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5">
       <c r="A92" s="21">
         <v>45477</v>
       </c>
@@ -2158,7 +2140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5">
       <c r="A93" s="21">
         <v>45484</v>
       </c>
@@ -2175,7 +2157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5">
       <c r="A94" s="21">
         <v>45491</v>
       </c>
@@ -2192,7 +2174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5">
       <c r="A95" s="21">
         <v>45498</v>
       </c>
@@ -2209,7 +2191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5">
       <c r="A96" s="21">
         <v>45505</v>
       </c>
@@ -2226,7 +2208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8">
       <c r="A97" s="21">
         <v>45512</v>
       </c>
@@ -2243,7 +2225,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8">
       <c r="A98" s="21">
         <v>45519</v>
       </c>
@@ -2260,7 +2242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:8" s="9" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" s="9" customFormat="1">
       <c r="A99" s="21">
         <v>45526</v>
       </c>
@@ -2280,7 +2262,7 @@
       <c r="G99" s="1"/>
       <c r="H99" s="1"/>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:8">
       <c r="A100" s="21">
         <v>45533</v>
       </c>
@@ -2297,7 +2279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:8" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" s="10" customFormat="1">
       <c r="A101" s="21">
         <v>45540</v>
       </c>
@@ -2317,7 +2299,7 @@
       <c r="G101" s="1"/>
       <c r="H101" s="1"/>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:8">
       <c r="A102" s="21">
         <v>45547</v>
       </c>
@@ -2334,7 +2316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:8">
       <c r="A103" s="21">
         <v>45554</v>
       </c>
@@ -2351,7 +2333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:8" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:8" s="10" customFormat="1">
       <c r="A104" s="21">
         <v>45561</v>
       </c>
@@ -2371,7 +2353,7 @@
       <c r="G104" s="1"/>
       <c r="H104" s="1"/>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:8">
       <c r="A105" s="21">
         <v>45568</v>
       </c>
@@ -2388,7 +2370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:8">
       <c r="A106" s="21">
         <v>45575</v>
       </c>
@@ -2405,7 +2387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:8">
       <c r="A107" s="21">
         <v>45582</v>
       </c>
@@ -2422,7 +2404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:8" s="11" customFormat="1">
       <c r="A108" s="21">
         <v>45589</v>
       </c>
@@ -2442,7 +2424,7 @@
       <c r="G108" s="1"/>
       <c r="H108" s="1"/>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8">
       <c r="A109" s="21">
         <v>45596</v>
       </c>
@@ -2459,7 +2441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:8" s="11" customFormat="1">
       <c r="A110" s="21">
         <v>45603</v>
       </c>
@@ -2479,7 +2461,7 @@
       <c r="G110" s="1"/>
       <c r="H110" s="1"/>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:8">
       <c r="A111" s="21">
         <v>45610</v>
       </c>
@@ -2499,7 +2481,7 @@
       <c r="G111" s="5"/>
       <c r="H111" s="5"/>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:8">
       <c r="A112" s="21">
         <v>45617</v>
       </c>
@@ -2516,7 +2498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:8" s="12" customFormat="1">
       <c r="A113" s="21">
         <v>45624</v>
       </c>
@@ -2536,7 +2518,7 @@
       <c r="G113" s="1"/>
       <c r="H113" s="1"/>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:8">
       <c r="A114" s="21">
         <v>45631</v>
       </c>
@@ -2553,7 +2535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:8" s="13" customFormat="1">
       <c r="A115" s="21">
         <v>45638</v>
       </c>
@@ -2573,7 +2555,7 @@
       <c r="G115" s="1"/>
       <c r="H115" s="1"/>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:8">
       <c r="A116" s="21">
         <v>45645</v>
       </c>
@@ -2590,7 +2572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:8">
       <c r="A117" s="21">
         <v>45659</v>
       </c>
@@ -2607,7 +2589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:8">
       <c r="A118" s="21">
         <v>45666</v>
       </c>
@@ -2624,7 +2606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:8">
       <c r="A119" s="21">
         <v>45673</v>
       </c>
@@ -2641,7 +2623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:8">
       <c r="A120" s="21">
         <v>45680</v>
       </c>
@@ -2658,7 +2640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:8" s="14" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:8" s="14" customFormat="1">
       <c r="A121" s="21">
         <v>45687</v>
       </c>
@@ -2678,7 +2660,7 @@
       <c r="G121" s="1"/>
       <c r="H121" s="1"/>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:8">
       <c r="A122" s="21">
         <v>45694</v>
       </c>
@@ -2695,7 +2677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:8" s="14" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:8" s="14" customFormat="1">
       <c r="A123" s="21">
         <v>45701</v>
       </c>
@@ -2715,7 +2697,7 @@
       <c r="G123" s="1"/>
       <c r="H123" s="1"/>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:8">
       <c r="A124" s="21">
         <v>45708</v>
       </c>
@@ -2732,7 +2714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:8" s="15" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:8" s="15" customFormat="1">
       <c r="A125" s="21">
         <v>45715</v>
       </c>
@@ -2752,7 +2734,7 @@
       <c r="G125" s="3"/>
       <c r="H125" s="3"/>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:8">
       <c r="A126" s="21">
         <v>45722</v>
       </c>
@@ -2771,7 +2753,7 @@
       <c r="F126" s="4"/>
       <c r="G126" s="5"/>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:8">
       <c r="A127" s="21">
         <v>45729</v>
       </c>
@@ -2788,7 +2770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:8" s="16" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:8" s="16" customFormat="1">
       <c r="A128" s="21">
         <v>45736</v>
       </c>
@@ -2808,7 +2790,7 @@
       <c r="G128" s="1"/>
       <c r="H128" s="1"/>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5">
       <c r="A129" s="21">
         <v>45743</v>
       </c>
@@ -2825,7 +2807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5">
       <c r="A130" s="21">
         <v>45750</v>
       </c>
@@ -2842,7 +2824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5">
       <c r="A131" s="21">
         <v>45757</v>
       </c>
@@ -2859,7 +2841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5">
       <c r="A132" s="21">
         <v>45764</v>
       </c>
@@ -2876,7 +2858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5">
       <c r="A133" s="21">
         <v>45771</v>
       </c>
@@ -2893,7 +2875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5">
       <c r="A134" s="21">
         <v>45778</v>
       </c>
@@ -2910,7 +2892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5">
       <c r="A135" s="21">
         <v>45785</v>
       </c>
@@ -2927,7 +2909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5">
       <c r="A136" s="21">
         <v>45792</v>
       </c>
@@ -2944,7 +2926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" s="17" customFormat="1">
       <c r="A137" s="21">
         <v>45799</v>
       </c>
@@ -2961,7 +2943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5">
       <c r="A138" s="21">
         <v>45806</v>
       </c>
@@ -2978,7 +2960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5">
       <c r="A139" s="21">
         <v>45813</v>
       </c>
@@ -2995,7 +2977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5">
       <c r="A140" s="21">
         <v>45820</v>
       </c>
@@ -3012,7 +2994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5">
       <c r="A141" s="21">
         <v>45827</v>
       </c>
@@ -3029,7 +3011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5">
       <c r="A142" s="21">
         <v>45834</v>
       </c>
@@ -3046,7 +3028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5">
       <c r="A143" s="21">
         <v>45841</v>
       </c>
@@ -3063,7 +3045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5">
       <c r="A144" s="21">
         <v>45848</v>
       </c>
@@ -3080,7 +3062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5">
       <c r="A145" s="21">
         <v>45855</v>
       </c>
@@ -3097,7 +3079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5">
       <c r="A146" s="21">
         <v>45862</v>
       </c>
@@ -3114,7 +3096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5">
       <c r="A147" s="21">
         <v>45869</v>
       </c>
@@ -3131,7 +3113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5">
       <c r="A148" s="21">
         <v>45876</v>
       </c>
@@ -3148,7 +3130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5">
       <c r="A149" s="21">
         <v>45883</v>
       </c>
@@ -3165,7 +3147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5">
       <c r="A150" s="21">
         <v>45890</v>
       </c>
@@ -3182,7 +3164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5">
       <c r="A151" s="21">
         <v>45897</v>
       </c>
@@ -3199,7 +3181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5">
       <c r="A152" s="21">
         <v>45904</v>
       </c>
@@ -3216,7 +3198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5">
       <c r="A153" s="21">
         <v>45911</v>
       </c>
@@ -3233,7 +3215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5">
       <c r="A154" s="21">
         <v>45918</v>
       </c>
@@ -3250,7 +3232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5">
       <c r="A155" s="21">
         <v>45925</v>
       </c>
@@ -3267,7 +3249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5">
       <c r="A156" s="21">
         <v>45932</v>
       </c>
@@ -3284,7 +3266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5">
       <c r="A157" s="21">
         <v>45939</v>
       </c>
@@ -3301,7 +3283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5">
       <c r="A158" s="21">
         <v>45946</v>
       </c>
@@ -3318,7 +3300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5">
       <c r="A159" s="21">
         <v>45953</v>
       </c>
@@ -3335,7 +3317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5">
       <c r="A160" s="21">
         <v>45960</v>
       </c>
@@ -3352,7 +3334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5">
       <c r="A161" s="21">
         <v>45967</v>
       </c>
@@ -3369,7 +3351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5">
       <c r="A162" s="21">
         <v>45974</v>
       </c>
@@ -3386,7 +3368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5">
       <c r="A163" s="21">
         <v>45981</v>
       </c>
@@ -3403,7 +3385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5">
       <c r="A164" s="21">
         <v>45988</v>
       </c>
@@ -3420,7 +3402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5">
       <c r="A165" s="21">
         <v>45995</v>
       </c>
@@ -3437,7 +3419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5">
       <c r="A166" s="21">
         <v>46002</v>
       </c>
@@ -3454,7 +3436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5">
       <c r="A167" s="21">
         <v>46009</v>
       </c>
@@ -3471,7 +3453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5">
       <c r="A168" s="21">
         <v>46014</v>
       </c>
@@ -3488,7 +3470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5">
       <c r="A169" s="21">
         <v>46030</v>
       </c>
@@ -3505,7 +3487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5">
       <c r="A170" s="21">
         <v>46037</v>
       </c>
@@ -3522,7 +3504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:5" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" s="18" customFormat="1">
       <c r="A171" s="21">
         <v>46044</v>
       </c>
@@ -3539,7 +3521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5">
       <c r="A172" s="21">
         <v>46051</v>
       </c>
@@ -3556,7 +3538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5">
       <c r="A173" s="21">
         <v>46058</v>
       </c>
@@ -3573,7 +3555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5">
       <c r="A174" s="21">
         <v>46065</v>
       </c>
@@ -3590,7 +3572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5">
       <c r="A175" s="21">
         <v>46072</v>
       </c>
@@ -3607,7 +3589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5">
       <c r="A176" s="21">
         <v>46079</v>
       </c>
@@ -3624,7 +3606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:8">
       <c r="A177" s="21">
         <v>46086</v>
       </c>
@@ -3641,7 +3623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:8">
       <c r="A178" s="21">
         <v>46093</v>
       </c>
@@ -3658,7 +3640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:8">
       <c r="A179" s="21">
         <v>46100</v>
       </c>
@@ -3675,7 +3657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:8">
       <c r="A180" s="21">
         <v>46107</v>
       </c>
@@ -3692,7 +3674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:8">
       <c r="A181" s="21">
         <v>46114</v>
       </c>
@@ -3709,7 +3691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:8">
       <c r="A182" s="21">
         <v>46121</v>
       </c>
@@ -3726,7 +3708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:8">
       <c r="A183" s="21">
         <v>46128</v>
       </c>
@@ -3743,7 +3725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:8">
       <c r="A184" s="21">
         <v>46135</v>
       </c>
@@ -3760,7 +3742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:8">
       <c r="A185" s="21">
         <v>46142</v>
       </c>
@@ -3777,7 +3759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:8">
       <c r="A186" s="21">
         <v>46149</v>
       </c>
@@ -3794,7 +3776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:8" s="19" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:8" s="19" customFormat="1">
       <c r="A187" s="21">
         <v>46156</v>
       </c>
@@ -3814,7 +3796,7 @@
       <c r="G187" s="1"/>
       <c r="H187" s="1"/>
     </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:8">
       <c r="A188" s="21">
         <v>46163</v>
       </c>
@@ -3831,7 +3813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:8">
       <c r="A189" s="21">
         <v>46170</v>
       </c>
@@ -3848,7 +3830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:8">
       <c r="A190" s="21">
         <v>46177</v>
       </c>
@@ -3865,7 +3847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:8">
       <c r="A191" s="21">
         <v>46184</v>
       </c>
@@ -3885,7 +3867,7 @@
       <c r="G191" s="5"/>
       <c r="H191" s="5"/>
     </row>
-    <row r="192" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:8">
       <c r="A192" s="21">
         <v>46191</v>
       </c>
@@ -3902,7 +3884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:8">
       <c r="A193" s="21">
         <v>46198</v>
       </c>
@@ -3919,7 +3901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:8">
       <c r="A194" s="21">
         <v>46205</v>
       </c>
@@ -3936,7 +3918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:8">
       <c r="A195" s="21">
         <v>46212</v>
       </c>
@@ -3953,7 +3935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:8">
       <c r="A196" s="21">
         <v>46219</v>
       </c>
@@ -3970,7 +3952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:8">
       <c r="A197" s="21">
         <v>46226</v>
       </c>
@@ -3987,7 +3969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:8">
       <c r="A198" s="21">
         <v>46233</v>
       </c>
@@ -4004,7 +3986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:8">
       <c r="A199" s="21">
         <v>46240</v>
       </c>
@@ -4021,7 +4003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:8">
       <c r="A200" s="21">
         <v>46247</v>
       </c>
@@ -4038,7 +4020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:8">
       <c r="A201" s="21">
         <v>46254</v>
       </c>
@@ -4055,7 +4037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:8">
       <c r="A202" s="21">
         <v>46261</v>
       </c>
@@ -4072,7 +4054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:8">
       <c r="A203" s="2">
         <v>46268</v>
       </c>
@@ -4089,7 +4071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:8" customFormat="1">
       <c r="A204" s="21">
         <v>46275</v>
       </c>
@@ -4106,7 +4088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:8">
       <c r="A205" s="2">
         <v>46282</v>
       </c>
@@ -4123,57 +4105,74 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A206" s="26">
+    <row r="206" spans="1:8">
+      <c r="A206" s="21">
         <v>46289</v>
       </c>
-      <c r="B206" s="27">
-        <v>7</v>
-      </c>
-      <c r="C206" s="26">
+      <c r="B206" s="22">
+        <v>7</v>
+      </c>
+      <c r="C206" s="21">
         <v>46296</v>
       </c>
-      <c r="D206" s="28">
+      <c r="D206" s="23">
         <v>128918</v>
       </c>
-      <c r="E206" s="29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A207" s="26">
+      <c r="E206" s="24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207" spans="1:8">
+      <c r="A207" s="21">
         <v>46296</v>
       </c>
-      <c r="B207" s="27">
-        <v>7</v>
-      </c>
-      <c r="C207" s="26">
+      <c r="B207" s="22">
+        <v>7</v>
+      </c>
+      <c r="C207" s="21">
         <v>46303</v>
       </c>
-      <c r="D207" s="28">
+      <c r="D207" s="23">
         <v>133441</v>
       </c>
-      <c r="E207" s="29">
-        <v>0</v>
-      </c>
-      <c r="F207" s="30"/>
-      <c r="G207" s="30"/>
-      <c r="H207" s="30"/>
-    </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E207" s="24">
+        <v>0</v>
+      </c>
+      <c r="F207" s="26"/>
+      <c r="G207" s="26"/>
+      <c r="H207" s="26"/>
+    </row>
+    <row r="208" spans="1:8">
       <c r="A208" s="2">
         <v>46303</v>
       </c>
-      <c r="B208" s="27">
+      <c r="B208" s="22">
         <v>7</v>
       </c>
       <c r="C208" s="2">
         <v>46310</v>
       </c>
-      <c r="D208" s="28">
+      <c r="D208" s="23">
         <v>132102</v>
       </c>
-      <c r="E208" s="29">
+      <c r="E208" s="24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" ht="15">
+      <c r="A209" s="2">
+        <v>46310</v>
+      </c>
+      <c r="B209" s="3">
+        <v>7</v>
+      </c>
+      <c r="C209" s="2">
+        <v>46317</v>
+      </c>
+      <c r="D209" s="23">
+        <v>140845</v>
+      </c>
+      <c r="E209" s="24">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data(gbp): daily refresh 2026-10-22T15:29Z
</commit_message>
<xml_diff>
--- a/logs/gbp/raw/boe_str.xlsx
+++ b/logs/gbp/raw/boe_str.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30610"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30611"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bankofenglandcouk.sharepoint.com/sites/SMD-Ops/Shared Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="6_{6357EF7E-F4D8-4EEB-8998-019A4B55854A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4039A544-9F63-40C1-8E4D-C2F4F752A111}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="6_{6357EF7E-F4D8-4EEB-8998-019A4B55854A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77B47EEC-3863-4441-A90A-C83DA6E0BCF1}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -574,7 +574,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:H209"/>
+  <dimension ref="A1:H210"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="17.5703125" style="1" customWidth="1"/>
@@ -4176,6 +4176,23 @@
         <v>0</v>
       </c>
     </row>
+    <row r="210" spans="1:5" ht="15">
+      <c r="A210" s="21">
+        <v>46317</v>
+      </c>
+      <c r="B210" s="22">
+        <v>7</v>
+      </c>
+      <c r="C210" s="21">
+        <v>46324</v>
+      </c>
+      <c r="D210" s="23">
+        <v>143083</v>
+      </c>
+      <c r="E210" s="24">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.98425196850393704" right="0.98425196850393704" top="0.98425196850393704" bottom="1.9842519685039399" header="0.98425196850393704" footer="0.98425196850393704"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
data(gbp): weekly refresh 2026-10-29T15:35Z
</commit_message>
<xml_diff>
--- a/logs/gbp/raw/boe_str.xlsx
+++ b/logs/gbp/raw/boe_str.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bankofenglandcouk.sharepoint.com/sites/SMD-Ops/Shared Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="6_{6357EF7E-F4D8-4EEB-8998-019A4B55854A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77B47EEC-3863-4441-A90A-C83DA6E0BCF1}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="6_{6357EF7E-F4D8-4EEB-8998-019A4B55854A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E87FC36B-D327-477F-A0A1-0FA4C3B5A6E6}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
     <numFmt numFmtId="165" formatCode="[$-10409]0.0"/>
     <numFmt numFmtId="166" formatCode="[$-10409]0.00"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -574,26 +574,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:H210"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
+  <dimension ref="A1:H211"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="24.140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="35.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.85546875" style="1"/>
+    <col min="1" max="1" width="17.54296875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="24.1796875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="35.453125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="9.1796875" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.81640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="13.7" customHeight="1">
+    <row r="1" spans="1:5" ht="13.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1"/>
       <c r="B1"/>
       <c r="C1"/>
       <c r="D1"/>
       <c r="E1"/>
     </row>
-    <row r="2" spans="1:5" ht="42">
+    <row r="2" spans="1:5" ht="42" x14ac:dyDescent="0.35">
       <c r="A2" s="20" t="s">
         <v>0</v>
       </c>
@@ -610,7 +610,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="21">
         <v>44840</v>
       </c>
@@ -627,7 +627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="21">
         <v>44847</v>
       </c>
@@ -644,7 +644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="21">
         <v>44854</v>
       </c>
@@ -661,7 +661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="21">
         <v>44861</v>
       </c>
@@ -678,7 +678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="21">
         <v>44868</v>
       </c>
@@ -695,7 +695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="21">
         <v>44875</v>
       </c>
@@ -712,7 +712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="21">
         <v>44882</v>
       </c>
@@ -729,7 +729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="21">
         <v>44889</v>
       </c>
@@ -746,7 +746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="21">
         <v>44896</v>
       </c>
@@ -763,7 +763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="21">
         <v>44903</v>
       </c>
@@ -780,7 +780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="21">
         <v>44910</v>
       </c>
@@ -797,7 +797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="21">
         <v>44917</v>
       </c>
@@ -814,7 +814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="21">
         <v>44931</v>
       </c>
@@ -831,7 +831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="21">
         <v>44938</v>
       </c>
@@ -848,7 +848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="21">
         <v>44945</v>
       </c>
@@ -865,7 +865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="21">
         <v>44952</v>
       </c>
@@ -882,7 +882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="21">
         <v>44959</v>
       </c>
@@ -899,7 +899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="21">
         <v>44966</v>
       </c>
@@ -916,7 +916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="21">
         <v>44973</v>
       </c>
@@ -933,7 +933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="21">
         <v>44980</v>
       </c>
@@ -950,7 +950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="21">
         <v>44987</v>
       </c>
@@ -967,7 +967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="21">
         <v>44994</v>
       </c>
@@ -984,7 +984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="21">
         <v>45001</v>
       </c>
@@ -1001,7 +1001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="21">
         <v>45008</v>
       </c>
@@ -1018,7 +1018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="21">
         <v>45015</v>
       </c>
@@ -1035,7 +1035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="21">
         <v>45022</v>
       </c>
@@ -1052,7 +1052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="21">
         <v>45029</v>
       </c>
@@ -1069,7 +1069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="21">
         <v>45036</v>
       </c>
@@ -1086,7 +1086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="21">
         <v>45043</v>
       </c>
@@ -1103,7 +1103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="21">
         <v>45050</v>
       </c>
@@ -1120,7 +1120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="21">
         <v>45057</v>
       </c>
@@ -1137,7 +1137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="21">
         <v>45064</v>
       </c>
@@ -1154,7 +1154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="21">
         <v>45071</v>
       </c>
@@ -1171,7 +1171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="21">
         <v>45078</v>
       </c>
@@ -1188,7 +1188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="21">
         <v>45085</v>
       </c>
@@ -1205,7 +1205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="21">
         <v>45092</v>
       </c>
@@ -1222,7 +1222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="21">
         <v>45099</v>
       </c>
@@ -1239,7 +1239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="21">
         <v>45106</v>
       </c>
@@ -1256,7 +1256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="21">
         <v>45113</v>
       </c>
@@ -1273,7 +1273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="21">
         <v>45120</v>
       </c>
@@ -1290,7 +1290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="21">
         <v>45127</v>
       </c>
@@ -1307,7 +1307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="21">
         <v>45134</v>
       </c>
@@ -1324,7 +1324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="21">
         <v>45141</v>
       </c>
@@ -1341,7 +1341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="21">
         <v>45148</v>
       </c>
@@ -1358,7 +1358,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="21">
         <v>45155</v>
       </c>
@@ -1375,7 +1375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="21">
         <v>45162</v>
       </c>
@@ -1392,7 +1392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="21">
         <v>45169</v>
       </c>
@@ -1409,7 +1409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="21">
         <v>45176</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="21">
         <v>45183</v>
       </c>
@@ -1443,7 +1443,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="21">
         <v>45190</v>
       </c>
@@ -1460,7 +1460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="21">
         <v>45197</v>
       </c>
@@ -1477,7 +1477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="21">
         <v>45204</v>
       </c>
@@ -1494,7 +1494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="21">
         <v>45211</v>
       </c>
@@ -1511,7 +1511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="21">
         <v>45218</v>
       </c>
@@ -1528,7 +1528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="21">
         <v>45225</v>
       </c>
@@ -1545,7 +1545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="21">
         <v>45232</v>
       </c>
@@ -1562,7 +1562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="21">
         <v>45239</v>
       </c>
@@ -1579,7 +1579,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:5" s="6" customFormat="1">
+    <row r="60" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A60" s="21">
         <v>45246</v>
       </c>
@@ -1596,7 +1596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="21">
         <v>45253</v>
       </c>
@@ -1613,7 +1613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="21">
         <v>45260</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="21">
         <v>45267</v>
       </c>
@@ -1647,7 +1647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:5" s="6" customFormat="1">
+    <row r="64" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A64" s="21">
         <v>45274</v>
       </c>
@@ -1664,7 +1664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="21">
         <v>45281</v>
       </c>
@@ -1681,7 +1681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:5" s="6" customFormat="1">
+    <row r="66" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A66" s="21">
         <v>45295</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="21">
         <v>45302</v>
       </c>
@@ -1715,7 +1715,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:5">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="21">
         <v>45309</v>
       </c>
@@ -1732,7 +1732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="21">
         <v>45316</v>
       </c>
@@ -1749,7 +1749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:5" s="7" customFormat="1">
+    <row r="70" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A70" s="21">
         <v>45323</v>
       </c>
@@ -1766,7 +1766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:5" s="7" customFormat="1">
+    <row r="71" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A71" s="21">
         <v>45330</v>
       </c>
@@ -1783,7 +1783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:5" s="7" customFormat="1">
+    <row r="72" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A72" s="21">
         <v>45337</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:5">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="21">
         <v>45344</v>
       </c>
@@ -1817,7 +1817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:5" s="7" customFormat="1">
+    <row r="74" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A74" s="21">
         <v>45351</v>
       </c>
@@ -1834,7 +1834,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:5">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="21">
         <v>45358</v>
       </c>
@@ -1851,7 +1851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:5">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="21">
         <v>45365</v>
       </c>
@@ -1868,7 +1868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="21">
         <v>45372</v>
       </c>
@@ -1885,7 +1885,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:5">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="21">
         <v>45379</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:5">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="21">
         <v>45386</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="21">
         <v>45393</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="21">
         <v>45400</v>
       </c>
@@ -1953,7 +1953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="21">
         <v>45407</v>
       </c>
@@ -1970,7 +1970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="21">
         <v>45414</v>
       </c>
@@ -1987,7 +1987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" s="8" customFormat="1">
+    <row r="84" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A84" s="21">
         <v>45421</v>
       </c>
@@ -2004,7 +2004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:5">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="21">
         <v>45428</v>
       </c>
@@ -2021,7 +2021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:5" s="8" customFormat="1">
+    <row r="86" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A86" s="21">
         <v>45435</v>
       </c>
@@ -2038,7 +2038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:5">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="21">
         <v>45442</v>
       </c>
@@ -2055,7 +2055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:5">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="21">
         <v>45449</v>
       </c>
@@ -2072,7 +2072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:5">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="21">
         <v>45456</v>
       </c>
@@ -2089,7 +2089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:5">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="21">
         <v>45463</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:5">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="21">
         <v>45470</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:5">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="21">
         <v>45477</v>
       </c>
@@ -2140,7 +2140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:5">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="21">
         <v>45484</v>
       </c>
@@ -2157,7 +2157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:5">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="21">
         <v>45491</v>
       </c>
@@ -2174,7 +2174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:5">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="21">
         <v>45498</v>
       </c>
@@ -2191,7 +2191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:5">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="21">
         <v>45505</v>
       </c>
@@ -2208,7 +2208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:8">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" s="21">
         <v>45512</v>
       </c>
@@ -2225,7 +2225,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:8">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A98" s="21">
         <v>45519</v>
       </c>
@@ -2242,7 +2242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:8" s="9" customFormat="1">
+    <row r="99" spans="1:8" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A99" s="21">
         <v>45526</v>
       </c>
@@ -2262,7 +2262,7 @@
       <c r="G99" s="1"/>
       <c r="H99" s="1"/>
     </row>
-    <row r="100" spans="1:8">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A100" s="21">
         <v>45533</v>
       </c>
@@ -2279,7 +2279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:8" s="10" customFormat="1">
+    <row r="101" spans="1:8" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A101" s="21">
         <v>45540</v>
       </c>
@@ -2299,7 +2299,7 @@
       <c r="G101" s="1"/>
       <c r="H101" s="1"/>
     </row>
-    <row r="102" spans="1:8">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A102" s="21">
         <v>45547</v>
       </c>
@@ -2316,7 +2316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:8">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A103" s="21">
         <v>45554</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:8" s="10" customFormat="1">
+    <row r="104" spans="1:8" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A104" s="21">
         <v>45561</v>
       </c>
@@ -2353,7 +2353,7 @@
       <c r="G104" s="1"/>
       <c r="H104" s="1"/>
     </row>
-    <row r="105" spans="1:8">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A105" s="21">
         <v>45568</v>
       </c>
@@ -2370,7 +2370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:8">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A106" s="21">
         <v>45575</v>
       </c>
@@ -2387,7 +2387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:8">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A107" s="21">
         <v>45582</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:8" s="11" customFormat="1">
+    <row r="108" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A108" s="21">
         <v>45589</v>
       </c>
@@ -2424,7 +2424,7 @@
       <c r="G108" s="1"/>
       <c r="H108" s="1"/>
     </row>
-    <row r="109" spans="1:8">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A109" s="21">
         <v>45596</v>
       </c>
@@ -2441,7 +2441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" s="11" customFormat="1">
+    <row r="110" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A110" s="21">
         <v>45603</v>
       </c>
@@ -2461,7 +2461,7 @@
       <c r="G110" s="1"/>
       <c r="H110" s="1"/>
     </row>
-    <row r="111" spans="1:8">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A111" s="21">
         <v>45610</v>
       </c>
@@ -2481,7 +2481,7 @@
       <c r="G111" s="5"/>
       <c r="H111" s="5"/>
     </row>
-    <row r="112" spans="1:8">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A112" s="21">
         <v>45617</v>
       </c>
@@ -2498,7 +2498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:8" s="12" customFormat="1">
+    <row r="113" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A113" s="21">
         <v>45624</v>
       </c>
@@ -2518,7 +2518,7 @@
       <c r="G113" s="1"/>
       <c r="H113" s="1"/>
     </row>
-    <row r="114" spans="1:8">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A114" s="21">
         <v>45631</v>
       </c>
@@ -2535,7 +2535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:8" s="13" customFormat="1">
+    <row r="115" spans="1:8" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A115" s="21">
         <v>45638</v>
       </c>
@@ -2555,7 +2555,7 @@
       <c r="G115" s="1"/>
       <c r="H115" s="1"/>
     </row>
-    <row r="116" spans="1:8">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A116" s="21">
         <v>45645</v>
       </c>
@@ -2572,7 +2572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:8">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A117" s="21">
         <v>45659</v>
       </c>
@@ -2589,7 +2589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:8">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A118" s="21">
         <v>45666</v>
       </c>
@@ -2606,7 +2606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:8">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A119" s="21">
         <v>45673</v>
       </c>
@@ -2623,7 +2623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:8">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A120" s="21">
         <v>45680</v>
       </c>
@@ -2640,7 +2640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:8" s="14" customFormat="1">
+    <row r="121" spans="1:8" s="14" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A121" s="21">
         <v>45687</v>
       </c>
@@ -2660,7 +2660,7 @@
       <c r="G121" s="1"/>
       <c r="H121" s="1"/>
     </row>
-    <row r="122" spans="1:8">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A122" s="21">
         <v>45694</v>
       </c>
@@ -2677,7 +2677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:8" s="14" customFormat="1">
+    <row r="123" spans="1:8" s="14" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A123" s="21">
         <v>45701</v>
       </c>
@@ -2697,7 +2697,7 @@
       <c r="G123" s="1"/>
       <c r="H123" s="1"/>
     </row>
-    <row r="124" spans="1:8">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A124" s="21">
         <v>45708</v>
       </c>
@@ -2714,7 +2714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:8" s="15" customFormat="1">
+    <row r="125" spans="1:8" s="15" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A125" s="21">
         <v>45715</v>
       </c>
@@ -2734,7 +2734,7 @@
       <c r="G125" s="3"/>
       <c r="H125" s="3"/>
     </row>
-    <row r="126" spans="1:8">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A126" s="21">
         <v>45722</v>
       </c>
@@ -2753,7 +2753,7 @@
       <c r="F126" s="4"/>
       <c r="G126" s="5"/>
     </row>
-    <row r="127" spans="1:8">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A127" s="21">
         <v>45729</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:8" s="16" customFormat="1">
+    <row r="128" spans="1:8" s="16" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A128" s="21">
         <v>45736</v>
       </c>
@@ -2790,7 +2790,7 @@
       <c r="G128" s="1"/>
       <c r="H128" s="1"/>
     </row>
-    <row r="129" spans="1:5">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="21">
         <v>45743</v>
       </c>
@@ -2807,7 +2807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:5">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="21">
         <v>45750</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:5">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="21">
         <v>45757</v>
       </c>
@@ -2841,7 +2841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:5">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="21">
         <v>45764</v>
       </c>
@@ -2858,7 +2858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:5">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="21">
         <v>45771</v>
       </c>
@@ -2875,7 +2875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:5">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="21">
         <v>45778</v>
       </c>
@@ -2892,7 +2892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:5">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="21">
         <v>45785</v>
       </c>
@@ -2909,7 +2909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:5">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="21">
         <v>45792</v>
       </c>
@@ -2926,7 +2926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:5" s="17" customFormat="1">
+    <row r="137" spans="1:5" s="17" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A137" s="21">
         <v>45799</v>
       </c>
@@ -2943,7 +2943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:5">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="21">
         <v>45806</v>
       </c>
@@ -2960,7 +2960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:5">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="21">
         <v>45813</v>
       </c>
@@ -2977,7 +2977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:5">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="21">
         <v>45820</v>
       </c>
@@ -2994,7 +2994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:5">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="21">
         <v>45827</v>
       </c>
@@ -3011,7 +3011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:5">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="21">
         <v>45834</v>
       </c>
@@ -3028,7 +3028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:5">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="21">
         <v>45841</v>
       </c>
@@ -3045,7 +3045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:5">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="21">
         <v>45848</v>
       </c>
@@ -3062,7 +3062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:5">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="21">
         <v>45855</v>
       </c>
@@ -3079,7 +3079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:5">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="21">
         <v>45862</v>
       </c>
@@ -3096,7 +3096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:5">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="21">
         <v>45869</v>
       </c>
@@ -3113,7 +3113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:5">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="21">
         <v>45876</v>
       </c>
@@ -3130,7 +3130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:5">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="21">
         <v>45883</v>
       </c>
@@ -3147,7 +3147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:5">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="21">
         <v>45890</v>
       </c>
@@ -3164,7 +3164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:5">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="21">
         <v>45897</v>
       </c>
@@ -3181,7 +3181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:5">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="21">
         <v>45904</v>
       </c>
@@ -3198,7 +3198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:5">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="21">
         <v>45911</v>
       </c>
@@ -3215,7 +3215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:5">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="21">
         <v>45918</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:5">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="21">
         <v>45925</v>
       </c>
@@ -3249,7 +3249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:5">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="21">
         <v>45932</v>
       </c>
@@ -3266,7 +3266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:5">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="21">
         <v>45939</v>
       </c>
@@ -3283,7 +3283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:5">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="21">
         <v>45946</v>
       </c>
@@ -3300,7 +3300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:5">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="21">
         <v>45953</v>
       </c>
@@ -3317,7 +3317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:5">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="21">
         <v>45960</v>
       </c>
@@ -3334,7 +3334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:5">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="21">
         <v>45967</v>
       </c>
@@ -3351,7 +3351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:5">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="21">
         <v>45974</v>
       </c>
@@ -3368,7 +3368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:5">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="21">
         <v>45981</v>
       </c>
@@ -3385,7 +3385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:5">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="21">
         <v>45988</v>
       </c>
@@ -3402,7 +3402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:5">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="21">
         <v>45995</v>
       </c>
@@ -3419,7 +3419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:5">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="21">
         <v>46002</v>
       </c>
@@ -3436,7 +3436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:5">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="21">
         <v>46009</v>
       </c>
@@ -3453,7 +3453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:5">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="21">
         <v>46014</v>
       </c>
@@ -3470,7 +3470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:5">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="21">
         <v>46030</v>
       </c>
@@ -3487,7 +3487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:5">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="21">
         <v>46037</v>
       </c>
@@ -3504,7 +3504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:5" s="18" customFormat="1">
+    <row r="171" spans="1:5" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A171" s="21">
         <v>46044</v>
       </c>
@@ -3521,7 +3521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:5">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="21">
         <v>46051</v>
       </c>
@@ -3538,7 +3538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:5">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="21">
         <v>46058</v>
       </c>
@@ -3555,7 +3555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:5">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="21">
         <v>46065</v>
       </c>
@@ -3572,7 +3572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:5">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="21">
         <v>46072</v>
       </c>
@@ -3589,7 +3589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:5">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="21">
         <v>46079</v>
       </c>
@@ -3606,7 +3606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:8">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A177" s="21">
         <v>46086</v>
       </c>
@@ -3623,7 +3623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:8">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A178" s="21">
         <v>46093</v>
       </c>
@@ -3640,7 +3640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:8">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A179" s="21">
         <v>46100</v>
       </c>
@@ -3657,7 +3657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:8">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A180" s="21">
         <v>46107</v>
       </c>
@@ -3674,7 +3674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:8">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A181" s="21">
         <v>46114</v>
       </c>
@@ -3691,7 +3691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:8">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A182" s="21">
         <v>46121</v>
       </c>
@@ -3708,7 +3708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:8">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A183" s="21">
         <v>46128</v>
       </c>
@@ -3725,7 +3725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:8">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A184" s="21">
         <v>46135</v>
       </c>
@@ -3742,7 +3742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:8">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A185" s="21">
         <v>46142</v>
       </c>
@@ -3759,7 +3759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:8">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A186" s="21">
         <v>46149</v>
       </c>
@@ -3776,7 +3776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:8" s="19" customFormat="1">
+    <row r="187" spans="1:8" s="19" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A187" s="21">
         <v>46156</v>
       </c>
@@ -3796,7 +3796,7 @@
       <c r="G187" s="1"/>
       <c r="H187" s="1"/>
     </row>
-    <row r="188" spans="1:8">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A188" s="21">
         <v>46163</v>
       </c>
@@ -3813,7 +3813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:8">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A189" s="21">
         <v>46170</v>
       </c>
@@ -3830,7 +3830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:8">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A190" s="21">
         <v>46177</v>
       </c>
@@ -3847,7 +3847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:8">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A191" s="21">
         <v>46184</v>
       </c>
@@ -3867,7 +3867,7 @@
       <c r="G191" s="5"/>
       <c r="H191" s="5"/>
     </row>
-    <row r="192" spans="1:8">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A192" s="21">
         <v>46191</v>
       </c>
@@ -3884,7 +3884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:8">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A193" s="21">
         <v>46198</v>
       </c>
@@ -3901,7 +3901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:8">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A194" s="21">
         <v>46205</v>
       </c>
@@ -3918,7 +3918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:8">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A195" s="21">
         <v>46212</v>
       </c>
@@ -3935,7 +3935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:8">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A196" s="21">
         <v>46219</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:8">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A197" s="21">
         <v>46226</v>
       </c>
@@ -3969,7 +3969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:8">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A198" s="21">
         <v>46233</v>
       </c>
@@ -3986,7 +3986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:8">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A199" s="21">
         <v>46240</v>
       </c>
@@ -4003,7 +4003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:8">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A200" s="21">
         <v>46247</v>
       </c>
@@ -4020,7 +4020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:8">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A201" s="21">
         <v>46254</v>
       </c>
@@ -4037,7 +4037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:8">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A202" s="21">
         <v>46261</v>
       </c>
@@ -4054,7 +4054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:8">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A203" s="2">
         <v>46268</v>
       </c>
@@ -4071,7 +4071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:8" customFormat="1">
+    <row r="204" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A204" s="21">
         <v>46275</v>
       </c>
@@ -4088,7 +4088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:8">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A205" s="2">
         <v>46282</v>
       </c>
@@ -4105,7 +4105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:8">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A206" s="21">
         <v>46289</v>
       </c>
@@ -4122,7 +4122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:8">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A207" s="21">
         <v>46296</v>
       </c>
@@ -4142,7 +4142,7 @@
       <c r="G207" s="26"/>
       <c r="H207" s="26"/>
     </row>
-    <row r="208" spans="1:8">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A208" s="2">
         <v>46303</v>
       </c>
@@ -4159,7 +4159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:5" ht="15">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A209" s="2">
         <v>46310</v>
       </c>
@@ -4176,7 +4176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:5" ht="15">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A210" s="21">
         <v>46317</v>
       </c>
@@ -4190,6 +4190,23 @@
         <v>143083</v>
       </c>
       <c r="E210" s="24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A211" s="21">
+        <v>46324</v>
+      </c>
+      <c r="B211" s="22">
+        <v>7</v>
+      </c>
+      <c r="C211" s="21">
+        <v>46331</v>
+      </c>
+      <c r="D211" s="23">
+        <v>139958</v>
+      </c>
+      <c r="E211" s="24">
         <v>0</v>
       </c>
     </row>

</xml_diff>